<commit_message>
Add file names to GWAS table
</commit_message>
<xml_diff>
--- a/results/13MANUSCRIPT_PLOTS_TABLES/tables/public_data_tables.xlsx
+++ b/results/13MANUSCRIPT_PLOTS_TABLES/tables/public_data_tables.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/darren/Documents/Post_doc/papers/2026_Nature_Genetics_eQTL/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/darren/Desktop/eQTL_study_2025/results/13MANUSCRIPT_PLOTS_TABLES/tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB27E7FA-865D-FA4A-A5E5-06FA28B20F2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51C26ED9-F2A4-9240-B553-D8A03B54EA80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13080" yWindow="2480" windowWidth="29540" windowHeight="18780" activeTab="2" xr2:uid="{E074B50A-D407-C345-94F9-F50AF47F467D}"/>
+    <workbookView xWindow="17800" yWindow="660" windowWidth="26560" windowHeight="19580" xr2:uid="{E074B50A-D407-C345-94F9-F50AF47F467D}"/>
   </bookViews>
   <sheets>
     <sheet name="GWAS" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="145">
   <si>
     <t>Name</t>
   </si>
@@ -185,12 +185,6 @@
     <t>https://figshare.com/ndownloader/files/51487022</t>
   </si>
   <si>
-    <t>https://figshare.com/ndownloader/articles/22564390/versions/1</t>
-  </si>
-  <si>
-    <t>https://figshare.com/ndownloader/articles/28707155/versions/4</t>
-  </si>
-  <si>
     <t>Schizophrenia GWAS sumstats</t>
   </si>
   <si>
@@ -347,9 +341,6 @@
     <t>PMID:26854917</t>
   </si>
   <si>
-    <t>Package to run TWAS (used to generate TWAS weights)</t>
-  </si>
-  <si>
     <t>cTWAS</t>
   </si>
   <si>
@@ -447,6 +438,42 @@
   </si>
   <si>
     <t>Python algorithm for batch-effect correction in single-cell RNA-seq data</t>
+  </si>
+  <si>
+    <t>Suite of tools for performing transcriptome-wide and regulome-wide association studies (used to generate TWAS weights)</t>
+  </si>
+  <si>
+    <t>bcftools</t>
+  </si>
+  <si>
+    <t>Utilities for variant calling and manipulating VCFs and BCFs</t>
+  </si>
+  <si>
+    <t>PMID:21903627</t>
+  </si>
+  <si>
+    <t>Filename</t>
+  </si>
+  <si>
+    <t>bip2024_eur_no23andMe.gz</t>
+  </si>
+  <si>
+    <t>ADHD2022_iPSYCH_deCODE_PGC.meta.gz</t>
+  </si>
+  <si>
+    <t>pgc-mdd2025_no23andMe-noUKBB_eur_v3-49-24-11.tsv.gz</t>
+  </si>
+  <si>
+    <t>daner_OCD_full_wo23andMe_190522.gz</t>
+  </si>
+  <si>
+    <t>PGC3_SCZ_wave3.european.autosome.public.v3.vcf.tsv.gz</t>
+  </si>
+  <si>
+    <t>https://figshare.com/ndownloader/files/53357735</t>
+  </si>
+  <si>
+    <t>https://figshare.com/ndownloader/files/40036684</t>
   </si>
 </sst>
 </file>
@@ -847,36 +874,40 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F485287C-4CDC-3840-8450-3028B5AF5602}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="56" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="4" max="4" width="43.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="56" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>38</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B2">
         <v>2022</v>
@@ -884,16 +915,19 @@
       <c r="C2" t="s">
         <v>39</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>45</v>
       </c>
       <c r="E2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+        <v>142</v>
+      </c>
+      <c r="F2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B3">
         <v>2025</v>
@@ -905,12 +939,15 @@
         <v>46</v>
       </c>
       <c r="E3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+      <c r="F3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B4">
         <v>2023</v>
@@ -918,16 +955,19 @@
       <c r="C4" t="s">
         <v>41</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="1" t="s">
         <v>47</v>
       </c>
       <c r="E4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+      <c r="F4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B5">
         <v>2023</v>
@@ -935,16 +975,19 @@
       <c r="C5" t="s">
         <v>43</v>
       </c>
-      <c r="D5" t="s">
-        <v>48</v>
-      </c>
-      <c r="E5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D5" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="F5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B6">
         <v>2025</v>
@@ -952,14 +995,23 @@
       <c r="C6" t="s">
         <v>44</v>
       </c>
-      <c r="D6" t="s">
-        <v>49</v>
+      <c r="D6" s="1" t="s">
+        <v>143</v>
       </c>
       <c r="E6" t="s">
-        <v>55</v>
+        <v>141</v>
+      </c>
+      <c r="F6" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{14F60109-2A2D-5647-B1E6-1C686F8AA6D4}"/>
+    <hyperlink ref="D4" r:id="rId2" xr:uid="{E9CA4202-F678-CC4E-937C-E4563718456C}"/>
+    <hyperlink ref="D6" r:id="rId3" xr:uid="{4EFF8025-198D-E64A-AF64-AC84B38F91D6}"/>
+    <hyperlink ref="D5" r:id="rId4" xr:uid="{D6E133B4-D905-5749-9E38-A2AED97C5641}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -978,16 +1030,16 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>38</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>42</v>
@@ -995,19 +1047,19 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>33</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="E2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -1015,16 +1067,16 @@
         <v>30</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C3" t="s">
         <v>31</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E3" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -1054,7 +1106,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -1087,7 +1139,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>17</v>
@@ -1101,12 +1153,12 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1116,7 +1168,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E09A8B3D-2146-5E44-9EB3-1997EF64E7CB}">
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.33203125" bestFit="1" customWidth="1"/>
@@ -1141,7 +1193,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>11</v>
@@ -1161,7 +1213,7 @@
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D3" t="s">
         <v>5</v>
@@ -1175,7 +1227,7 @@
         <v>19</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D4" t="s">
         <v>18</v>
@@ -1189,7 +1241,7 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D5" t="s">
         <v>21</v>
@@ -1203,10 +1255,10 @@
         <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D6" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -1217,7 +1269,7 @@
         <v>2.4</v>
       </c>
       <c r="C7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D7" t="s">
         <v>25</v>
@@ -1231,10 +1283,10 @@
         <v>1.9</v>
       </c>
       <c r="C8" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D8" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -1245,10 +1297,10 @@
         <v>2</v>
       </c>
       <c r="C9" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D9" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -1256,10 +1308,10 @@
         <v>28</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D10" t="s">
         <v>29</v>
@@ -1270,13 +1322,13 @@
         <v>32</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D11" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -1287,10 +1339,10 @@
         <v>35</v>
       </c>
       <c r="C12" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D12" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
@@ -1301,163 +1353,177 @@
         <v>37</v>
       </c>
       <c r="C13" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D13" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D14" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C15" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D15" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C16" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D16" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C17" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D17" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>85</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D18" t="s">
         <v>87</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="D18" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C19" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D19" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>89</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C20" t="s">
         <v>91</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="D20" t="s">
         <v>92</v>
-      </c>
-      <c r="C20" t="s">
-        <v>93</v>
-      </c>
-      <c r="D20" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
+        <v>94</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="C21" t="s">
         <v>96</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="D21" t="s">
         <v>97</v>
-      </c>
-      <c r="C21" t="s">
-        <v>98</v>
-      </c>
-      <c r="D21" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C22" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D22" t="s">
-        <v>102</v>
+        <v>133</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B23" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="C23" t="s">
         <v>118</v>
       </c>
-      <c r="C23" t="s">
-        <v>121</v>
-      </c>
       <c r="D23" s="5" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B24" s="7">
         <v>0.1</v>
       </c>
       <c r="C24" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D24" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>134</v>
+      </c>
+      <c r="B25" s="7">
+        <v>1.9</v>
+      </c>
+      <c r="C25" t="s">
+        <v>136</v>
+      </c>
+      <c r="D25" t="s">
         <v>135</v>
       </c>
     </row>

</xml_diff>